<commit_message>
Implemented dynamic formula application in CAPEX sheet for fuel markets (LPG, Electricity)
</commit_message>
<xml_diff>
--- a/backend/technoeconomic-inputs/technoeconomic-inputs-template.xlsx
+++ b/backend/technoeconomic-inputs/technoeconomic-inputs-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8954da175e61d5af/Escritorio/IIT/NICCP-AI/backend/technoeconomic-inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="10_ncr:20000_{4F2B366B-AA2F-4F18-863E-957538EF6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F4AD43A5-47E6-4B40-8048-7A32343975FD}"/>
+  <xr:revisionPtr revIDLastSave="65" documentId="10_ncr:20000_{4F2B366B-AA2F-4F18-863E-957538EF6F0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{32BF4B22-4E42-44BC-BDC6-3DEBC3125F0E}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Electricity" sheetId="2" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="492" uniqueCount="54">
   <si>
     <t>Units</t>
   </si>
@@ -175,16 +175,31 @@
     <t>CAPEX - OFF GRID</t>
   </si>
   <si>
-    <t>CAPEX - Heat</t>
-  </si>
-  <si>
-    <t>OPEX - Heat</t>
-  </si>
-  <si>
     <t>CAPEX - UPSTREAM</t>
   </si>
   <si>
     <t>OPEX - UPSTREAM</t>
+  </si>
+  <si>
+    <t>GRID</t>
+  </si>
+  <si>
+    <t>OFF GRID</t>
+  </si>
+  <si>
+    <t>LOCAL</t>
+  </si>
+  <si>
+    <t>UPSTREAM</t>
+  </si>
+  <si>
+    <t>CAPEX - HEAT</t>
+  </si>
+  <si>
+    <t>OPEX - HEAT</t>
+  </si>
+  <si>
+    <t>HEAT</t>
   </si>
 </sst>
 </file>
@@ -421,7 +436,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -520,6 +535,9 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -536,6 +554,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1560,7 +1582,7 @@
     </row>
     <row r="8" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="8" t="s">
-        <v>16</v>
+        <v>47</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>10</v>
@@ -2202,7 +2224,7 @@
     </row>
     <row r="14" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="13" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>10</v>
@@ -2523,7 +2545,7 @@
     </row>
     <row r="17" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="31" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="B17" s="6" t="s">
         <v>14</v>
@@ -2630,7 +2652,7 @@
     </row>
     <row r="18" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="32" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="B18" s="7" t="s">
         <v>15</v>
@@ -2737,7 +2759,7 @@
     </row>
     <row r="19" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="14" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="B19" s="7" t="s">
         <v>10</v>
@@ -3608,7 +3630,7 @@
     </row>
     <row r="8" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="8" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>23</v>
@@ -3715,7 +3737,7 @@
     </row>
     <row r="9" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="13" t="s">
-        <v>16</v>
+        <v>49</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>24</v>
@@ -3929,7 +3951,7 @@
     </row>
     <row r="11" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B11" s="6" t="s">
         <v>19</v>
@@ -4036,7 +4058,7 @@
     </row>
     <row r="12" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="6" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="B12" s="6" t="s">
         <v>20</v>
@@ -4143,7 +4165,7 @@
     </row>
     <row r="13" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B13" s="7" t="s">
         <v>21</v>
@@ -4250,7 +4272,7 @@
     </row>
     <row r="14" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B14" s="7" t="s">
         <v>22</v>
@@ -4291,7 +4313,7 @@
     </row>
     <row r="15" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="7" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B15" s="7" t="s">
         <v>26</v>
@@ -4397,6 +4419,9 @@
       </c>
     </row>
     <row r="16" spans="1:35" ht="16" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A16" s="33" t="s">
+        <v>50</v>
+      </c>
       <c r="B16" s="7" t="s">
         <v>10</v>
       </c>

</xml_diff>